<commit_message>
Add Figure 4b and update figure names
</commit_message>
<xml_diff>
--- a/data/analysis/Figure-4_source-data.xlsx
+++ b/data/analysis/Figure-4_source-data.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure-4a" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure-4b" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure-4c" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Figure-3a" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Figure-3b" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Figure-4a" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Figure-4b" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -670,7 +671,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -692,7 +693,7 @@
         <v>2030</v>
       </c>
       <c r="G7" t="n">
-        <v>21.34924951171876</v>
+        <v>20.58626489257813</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -708,7 +709,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -730,7 +731,7 @@
         <v>2030</v>
       </c>
       <c r="G8" t="n">
-        <v>20.58626489257813</v>
+        <v>21.34924951171876</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -822,7 +823,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -844,7 +845,7 @@
         <v>2030</v>
       </c>
       <c r="G11" t="n">
-        <v>11.91799999999999</v>
+        <v>14.739</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -860,7 +861,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -882,7 +883,7 @@
         <v>2030</v>
       </c>
       <c r="G12" t="n">
-        <v>14.739</v>
+        <v>11.91799999999999</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -974,7 +975,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -996,7 +997,7 @@
         <v>2030</v>
       </c>
       <c r="G15" t="n">
-        <v>95.31103558132344</v>
+        <v>0</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1012,7 +1013,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1034,7 +1035,7 @@
         <v>2030</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>95.31103558132344</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1126,7 +1127,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1164,7 +1165,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1278,7 +1279,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1300,7 +1301,7 @@
         <v>2030</v>
       </c>
       <c r="G23" t="n">
-        <v>256.459241</v>
+        <v>269.7368224</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1316,7 +1317,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1338,7 +1339,7 @@
         <v>2030</v>
       </c>
       <c r="G24" t="n">
-        <v>269.7368224</v>
+        <v>256.459241</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1430,7 +1431,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1452,7 +1453,7 @@
         <v>2030</v>
       </c>
       <c r="G27" t="n">
-        <v>23.1029235146622</v>
+        <v>13.3648982490056</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1468,7 +1469,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1490,7 +1491,7 @@
         <v>2030</v>
       </c>
       <c r="G28" t="n">
-        <v>13.3648982490056</v>
+        <v>23.1029235146622</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1696,7 +1697,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1718,7 +1719,7 @@
         <v>2040</v>
       </c>
       <c r="G34" t="n">
-        <v>217.219125</v>
+        <v>209.0166328125</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -1734,7 +1735,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1756,7 +1757,7 @@
         <v>2040</v>
       </c>
       <c r="G35" t="n">
-        <v>209.0166328125</v>
+        <v>217.219125</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -1848,7 +1849,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1870,7 +1871,7 @@
         <v>2040</v>
       </c>
       <c r="G38" t="n">
-        <v>288.866</v>
+        <v>290.279</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -1886,7 +1887,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1908,7 +1909,7 @@
         <v>2040</v>
       </c>
       <c r="G39" t="n">
-        <v>290.279</v>
+        <v>288.866</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -2000,7 +2001,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2022,7 +2023,7 @@
         <v>2040</v>
       </c>
       <c r="G42" t="n">
-        <v>495.8784542725003</v>
+        <v>323.231180579626</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2038,7 +2039,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2060,7 +2061,7 @@
         <v>2040</v>
       </c>
       <c r="G43" t="n">
-        <v>323.231180579626</v>
+        <v>495.8784542725003</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2152,7 +2153,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2174,7 +2175,7 @@
         <v>2040</v>
       </c>
       <c r="G46" t="n">
-        <v>250.22777634</v>
+        <v>251.424997465</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2190,7 +2191,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2212,7 +2213,7 @@
         <v>2040</v>
       </c>
       <c r="G47" t="n">
-        <v>251.424997465</v>
+        <v>250.22777634</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -2304,7 +2305,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2326,7 +2327,7 @@
         <v>2040</v>
       </c>
       <c r="G50" t="n">
-        <v>757.4503447</v>
+        <v>722.7477461</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -2342,7 +2343,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2364,7 +2365,7 @@
         <v>2040</v>
       </c>
       <c r="G51" t="n">
-        <v>722.7477461</v>
+        <v>757.4503447</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -2456,7 +2457,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2478,7 +2479,7 @@
         <v>2040</v>
       </c>
       <c r="G54" t="n">
-        <v>112.716517831094</v>
+        <v>79.4029463553114</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -2494,7 +2495,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2516,7 +2517,7 @@
         <v>2040</v>
       </c>
       <c r="G55" t="n">
-        <v>79.4029463553114</v>
+        <v>112.716517831094</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -2722,7 +2723,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2744,7 +2745,7 @@
         <v>2050</v>
       </c>
       <c r="G61" t="n">
-        <v>236.046296875</v>
+        <v>222.15284375</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -2760,7 +2761,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2782,7 +2783,7 @@
         <v>2050</v>
       </c>
       <c r="G62" t="n">
-        <v>222.15284375</v>
+        <v>236.046296875</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -2874,7 +2875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2896,7 +2897,7 @@
         <v>2050</v>
       </c>
       <c r="G65" t="n">
-        <v>454.298</v>
+        <v>468.311</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -2912,7 +2913,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2934,7 +2935,7 @@
         <v>2050</v>
       </c>
       <c r="G66" t="n">
-        <v>468.311</v>
+        <v>454.298</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -3026,7 +3027,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3048,7 +3049,7 @@
         <v>2050</v>
       </c>
       <c r="G69" t="n">
-        <v>1066.820812525584</v>
+        <v>749.5352971884492</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -3064,7 +3065,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3086,7 +3087,7 @@
         <v>2050</v>
       </c>
       <c r="G70" t="n">
-        <v>749.5352971884492</v>
+        <v>1066.820812525584</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -3178,7 +3179,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3200,7 +3201,7 @@
         <v>2050</v>
       </c>
       <c r="G73" t="n">
-        <v>347.6144401225</v>
+        <v>345.712703185</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -3216,7 +3217,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3238,7 +3239,7 @@
         <v>2050</v>
       </c>
       <c r="G74" t="n">
-        <v>345.712703185</v>
+        <v>347.6144401225</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -3330,7 +3331,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3352,7 +3353,7 @@
         <v>2050</v>
       </c>
       <c r="G77" t="n">
-        <v>889.3851582999999</v>
+        <v>799.0676647</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -3368,7 +3369,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3390,7 +3391,7 @@
         <v>2050</v>
       </c>
       <c r="G78" t="n">
-        <v>799.0676647</v>
+        <v>889.3851582999999</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -3482,7 +3483,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>NetZero|LimCCS</t>
+          <t>NetZero|LimNuc</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3504,7 +3505,7 @@
         <v>2050</v>
       </c>
       <c r="G81" t="n">
-        <v>150.941843400535</v>
+        <v>166.825260165843</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -3520,7 +3521,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>NetZero|LimNuc</t>
+          <t>NetZero|LimCCS</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3542,7 +3543,7 @@
         <v>2050</v>
       </c>
       <c r="G82" t="n">
-        <v>166.825260165843</v>
+        <v>150.941843400535</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -9730,4 +9731,535 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>demand_response</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>spatial_resolution</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>flexible_generation</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>flexible_demand</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>hydrogen</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>spatial</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>curtailment</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>breadth</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>intensity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AIM-T</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NetZero</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>EU27 &amp; UK (*)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0.02594353154081003</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.07639607307698748</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1129961552551351</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.06851521209347103</v>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>0.02410710067357368</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.812558199619114</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.05132634543999622</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>IMAGE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NetZero</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EU27 &amp; UK (*)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.05250748021644651</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.1133602172471355</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.001490669298023223</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.000199791447889586</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.09056685220299404</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.6072868395761468</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.04302083506874815</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MEESA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NetZero</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EU27 &amp; UK (*)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0.1474986951620031</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.1190358090762738</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>0.06354137032470386</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.0001740416829830744</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.06256064843883784</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.7368658530758457</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.06546842744746695</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MESSAGEix</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NetZero</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EU27 &amp; UK (*)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>0.2014597615313616</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.2557301058191569</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.09629329410526999</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.004914625419535361</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.09147609550672357</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0006969413051949144</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.7439022645626518</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.1084284706145404</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PROMETHEUS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NetZero</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EU27 &amp; UK (*)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>0.1086944241736598</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.1309323725107457</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.3844460402167717</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.03993779944740092</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>REMIND</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NetZero</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EU27 &amp; UK (*)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0.1859719134422717</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.06908792935613303</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.03359520937577645</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.09911953901321338</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.6810909675962894</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.0646290985312324</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TIAM-ECN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NetZero</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>EU27 &amp; UK (*)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>0.119013966267267</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.01175293069312545</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.004668142155740415</v>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.2465621140950592</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.02257250651935548</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WITCH</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NetZero</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EU27 &amp; UK (*)</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Very low</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>0.04125586027473353</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.08122709127546655</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.1864066046741709</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>0.206488427639257</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.6851503976660761</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.08589633064393799</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Apply changes after adding new modules (solar-storage)
</commit_message>
<xml_diff>
--- a/data/analysis/Figure-4_source-data.xlsx
+++ b/data/analysis/Figure-4_source-data.xlsx
@@ -9173,7 +9173,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>r_storage_power_over_total_capacity</t>
+          <t>r_storage_power_over_peak_load</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -9262,7 +9262,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.02594353154081003</v>
+        <v>0.07687806618934163</v>
       </c>
       <c r="H2" t="n">
         <v>0.07639607307698748</v>
@@ -9322,7 +9322,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.05250748021644651</v>
+        <v>0.2482756922094443</v>
       </c>
       <c r="H3" t="n">
         <v>0.1133602172471355</v>
@@ -9388,7 +9388,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.1474986951620031</v>
+        <v>0.5061264211111115</v>
       </c>
       <c r="H4" t="n">
         <v>0.1190358090762738</v>
@@ -9452,7 +9452,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.2014597615313616</v>
+        <v>0.630851794825963</v>
       </c>
       <c r="H5" t="n">
         <v>0.2557301058191569</v>
@@ -9518,7 +9518,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.1086944241736598</v>
+        <v>0.4068465390988477</v>
       </c>
       <c r="H6" t="n">
         <v>0.1309323725107457</v>
@@ -9570,7 +9570,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.1859719134422717</v>
+        <v>0.7832486522686055</v>
       </c>
       <c r="H7" t="n">
         <v>0.06908792935613303</v>
@@ -9696,7 +9696,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.04125586027473353</v>
+        <v>0.09079633101343609</v>
       </c>
       <c r="H9" t="n">
         <v>0.08122709127546655</v>
@@ -9849,7 +9849,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.02594353154081003</v>
+        <v>0.07687806618934163</v>
       </c>
       <c r="H2" t="n">
         <v>0.07639607307698748</v>
@@ -9868,10 +9868,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="N2" t="n">
-        <v>0.812558199619114</v>
+        <v>0.8487568811235685</v>
       </c>
       <c r="O2" t="n">
-        <v>0.05132634543999622</v>
+        <v>0.05981543454808482</v>
       </c>
     </row>
     <row r="3">
@@ -9904,7 +9904,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.05250748021644651</v>
+        <v>0.2482756922094443</v>
       </c>
       <c r="H3" t="n">
         <v>0.1133602172471355</v>
@@ -9925,10 +9925,10 @@
         <v>0.5</v>
       </c>
       <c r="N3" t="n">
-        <v>0.6072868395761468</v>
+        <v>0.5694262108491379</v>
       </c>
       <c r="O3" t="n">
-        <v>0.04302083506874815</v>
+        <v>0.07564887040091445</v>
       </c>
     </row>
     <row r="4">
@@ -9961,7 +9961,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.1474986951620031</v>
+        <v>0.5061264211111115</v>
       </c>
       <c r="H4" t="n">
         <v>0.1190358090762738</v>
@@ -9980,10 +9980,10 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="N4" t="n">
-        <v>0.7368658530758457</v>
+        <v>0.5446338012825681</v>
       </c>
       <c r="O4" t="n">
-        <v>0.06546842744746695</v>
+        <v>0.1252397151056517</v>
       </c>
     </row>
     <row r="5">
@@ -10016,7 +10016,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.2014597615313616</v>
+        <v>0.630851794825963</v>
       </c>
       <c r="H5" t="n">
         <v>0.2557301058191569</v>
@@ -10037,10 +10037,10 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="N5" t="n">
-        <v>0.7439022645626518</v>
+        <v>0.6189841485329652</v>
       </c>
       <c r="O5" t="n">
-        <v>0.1084284706145404</v>
+        <v>0.179993809496974</v>
       </c>
     </row>
     <row r="6">
@@ -10073,7 +10073,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.1086944241736598</v>
+        <v>0.4068465390988477</v>
       </c>
       <c r="H6" t="n">
         <v>0.1309323725107457</v>
@@ -10088,10 +10088,10 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="N6" t="n">
-        <v>0.3844460402167717</v>
+        <v>0.3097767569210332</v>
       </c>
       <c r="O6" t="n">
-        <v>0.03993779944740092</v>
+        <v>0.08962981860159891</v>
       </c>
     </row>
     <row r="7">
@@ -10124,7 +10124,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.1859719134422717</v>
+        <v>0.7832486522686055</v>
       </c>
       <c r="H7" t="n">
         <v>0.06908792935613303</v>
@@ -10145,10 +10145,10 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="N7" t="n">
-        <v>0.6810909675962894</v>
+        <v>0.3990157790603294</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0646290985312324</v>
+        <v>0.1641752216689547</v>
       </c>
     </row>
     <row r="8">
@@ -10234,7 +10234,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.04125586027473353</v>
+        <v>0.09079633101343609</v>
       </c>
       <c r="H9" t="n">
         <v>0.08122709127546655</v>
@@ -10253,10 +10253,10 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="N9" t="n">
-        <v>0.6851503976660761</v>
+        <v>0.7291181771086733</v>
       </c>
       <c r="O9" t="n">
-        <v>0.08589633064393799</v>
+        <v>0.0941530757670551</v>
       </c>
     </row>
   </sheetData>

</xml_diff>